<commit_message>
Runbook: add standing Helverin/Crusader Bondsman reminder to the cheat-sheet
Every-turn reminder in the rules cheat-sheet (prints ahead of all battle plans):
keep the Helverin in the Crusader's Bondsman range for +1 to hit (BS2+ autocannons),
hold it back as the safe OC6 home anchor + Suppression. Regenerated all 3 docs.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Reports & Plans/LSO-Knights-List-and-Analysis.xlsx
+++ b/docs/Reports & Plans/LSO-Knights-List-and-Analysis.xlsx
@@ -1968,7 +1968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2102,15 +2102,27 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>Helverin Bondsman (EVERY TURN)</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Keep the Armiger Helverin within Bondsman range of the KNIGHT CRUSADER -&gt; Crusader's Duty = +1 to hit = BS2+ on its 8 autocannon shots (48"). It is your SAFE backfield/home OC6 anchor + Suppression (-1 to hit its target) -- do NOT push it forward, and don't let it drift out of the Crusader's bond.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>MINDSET</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Knights are 'always outnumbered, rarely outgunned.' At a 300+ GT, START every hard matchup from the EXPECTATION OF A LOSS and hunt the HEIST. Model the opponent playing OPTIMALLY. Realistic goal: a strong POSITIVE record + steal a couple you shouldn't win — not winning the event. The 2 Volcano lances win the shooting phase; the Lancer wins the melee phase you can't tank; you win the game on the mission (out-OC where you can).</t>
         </is>
@@ -2118,9 +2130,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A13:B13"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A15:B15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>